<commit_message>
Refactor flow to read Xetra-specific statuses and add video demo script
</commit_message>
<xml_diff>
--- a/tests/runs/run_1/evidence_ReportTypeA.xlsx
+++ b/tests/runs/run_1/evidence_ReportTypeA.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReportTypeA Evidence" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Xetra Trades" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,21 +28,37 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="0000335B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00D9383A"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0000335B"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +71,18 @@
         <bgColor rgb="0000335B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+        <bgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -65,26 +93,34 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,118 +486,1098 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Date</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Report Type</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Coverage Period</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Violation Marker</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Validation Status</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Threshold1</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Threshold2</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Threshold3</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Threshold4</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Breach Details</t>
+          <t>Xetra Daily Trading Report — 2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>20260530</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>ReportTypeA</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Daily</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+          <t>Report ID: XETRA-DA-20260530  |  Venue: XETR  |  Member: FRAUAS01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>TradeID</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ExecutionTime</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ISIN</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Instrument</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>OrderType</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>TraderID</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>DayViol</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>ViolationDetails</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00001</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>DE0007236101</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>165.58</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Stop-Limit</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>T-1042</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00002</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>12:32:38</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>DE0007236101</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>160.74</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>T-5023</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Late trade booking — execution not reported within T+0 window</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>Violation</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Threshold breach: Threshold2 (16 &lt; 50)</t>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00003</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>09:48:51</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>DE000A1EWWW0</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>adidas AG</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>223.48</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>T-6091</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00004</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>10:05:24</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>DE000BASF111</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>BASF SE</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>44.94</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>T-3011</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Wash trade suspicion — offsetting buy/sell within 60 seconds</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>Violation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00005</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>10:35:18</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>DE000DTR0CK8</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Daimler Truck Holding</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>41.75</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>T-3011</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00006</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>13:05:54</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>DE000DTR0CK8</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Daimler Truck Holding</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>38.32</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>T-3011</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00007</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>11:23:22</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>DE0007236101</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>175.89</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>T-4055</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00008</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>11:29:24</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>DE0005140008</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Deutsche Bank AG</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>16.60</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>T-6091</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00009</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>12:52:02</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>DE0008430026</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Münchener Rück</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>473.71</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>T-6091</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00010</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>14:13:41</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>DE000BASF111</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>BASF SE</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>51.22</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Stop-Limit</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>T-3011</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00011</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>17:34:16</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>DE0008430026</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Münchener Rück</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>445.59</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Stop-Limit</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>T-4055</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00012</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>17:31:05</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>DE000BASF111</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>BASF SE</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>44.97</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>T-5023</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00013</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>15:38:29</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>DE0007236101</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>174.91</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>T-2087</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00014</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>10:18:27</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>DE0005557508</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Deutsche Telekom AG</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>27.07</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>T-1042</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>XTR-20260530-00015</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>13:53:40</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>DE0007164600</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>197.69</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>T-6091</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Total Trades: 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Total Volume: EUR 865137.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Violations Found: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Overall Status: Violation</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>